<commit_message>
Format teks untuk NPWP, agar +15 dapat terbaca
</commit_message>
<xml_diff>
--- a/Dapur/Template_v.1.6.1.xlsx
+++ b/Dapur/Template_v.1.6.1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adminF\Downloads\Auto-Input-XML-Pajak-Coretax-1.2.3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adminF\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC76576-79E6-4DCD-833D-13792D7B4033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{194DB5F2-BE09-4247-85EA-0C394ED32F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2942,7 +2942,7 @@
     <t>Initial</t>
   </si>
   <si>
-    <t>00123456789</t>
+    <t>0012345678999000</t>
   </si>
 </sst>
 </file>
@@ -3125,7 +3125,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3204,6 +3204,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3620,7 +3623,7 @@
     <col min="8" max="8" width="11" customWidth="1"/>
     <col min="9" max="9" width="18.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="29.7109375" customWidth="1"/>
-    <col min="11" max="11" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.140625" style="38" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="27.7109375" customWidth="1"/>
     <col min="13" max="13" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="29.140625" customWidth="1"/>
@@ -3631,10 +3634,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="38"/>
+      <c r="B1" s="41"/>
       <c r="C1" s="9" t="s">
         <v>840</v>
       </c>
@@ -3675,7 +3678,7 @@
       <c r="J3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="39" t="s">
         <v>6</v>
       </c>
       <c r="L3" s="4" t="s">
@@ -3711,7 +3714,7 @@
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
       <c r="J4" s="11"/>
-      <c r="K4" s="1"/>
+      <c r="K4" s="40"/>
       <c r="L4" s="9"/>
       <c r="M4" s="9"/>
       <c r="N4" s="9"/>
@@ -3901,10 +3904,10 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="39"/>
+      <c r="B2" s="42"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -3923,10 +3926,10 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="39" t="s">
+      <c r="A5" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="39"/>
+      <c r="B5" s="42"/>
     </row>
     <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
@@ -4009,10 +4012,10 @@
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="39" t="s">
+      <c r="A16" s="42" t="s">
         <v>131</v>
       </c>
-      <c r="B16" s="39"/>
+      <c r="B16" s="42"/>
     </row>
     <row r="17" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
@@ -4047,10 +4050,10 @@
       </c>
     </row>
     <row r="21" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="40" t="s">
+      <c r="A21" s="43" t="s">
         <v>499</v>
       </c>
-      <c r="B21" s="40"/>
+      <c r="B21" s="43"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
@@ -4416,10 +4419,10 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="44" t="s">
         <v>828</v>
       </c>
-      <c r="B2" s="42"/>
+      <c r="B2" s="45"/>
       <c r="C2" s="37" t="s">
         <v>829</v>
       </c>
@@ -4769,10 +4772,10 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="44" t="s">
         <v>830</v>
       </c>
-      <c r="B2" s="42"/>
+      <c r="B2" s="45"/>
       <c r="C2" s="37" t="s">
         <v>831</v>
       </c>
@@ -5092,10 +5095,10 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="42" t="s">
         <v>139</v>
       </c>
-      <c r="B2" s="39"/>
+      <c r="B2" s="42"/>
     </row>
     <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
@@ -7170,10 +7173,10 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="46" t="s">
         <v>578</v>
       </c>
-      <c r="B2" s="43"/>
+      <c r="B2" s="46"/>
       <c r="C2" s="21"/>
       <c r="D2" s="19"/>
     </row>
@@ -7424,10 +7427,10 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="43" t="s">
+      <c r="A21" s="46" t="s">
         <v>579</v>
       </c>
-      <c r="B21" s="43"/>
+      <c r="B21" s="46"/>
       <c r="C21" s="21"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>